<commit_message>
Set vehicle logit function to use cost per thing*mile rather than NPV of lifetime cost; draft settings for TTLE and TTS
</commit_message>
<xml_diff>
--- a/InputData/trans/TTLE/Transportation Technology Logit Exponents.xlsx
+++ b/InputData/trans/TTLE/Transportation Technology Logit Exponents.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\trans\TTLE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6CC5EDA-16E8-45C6-851B-8000B937503F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2886E2FB-015D-47A1-A529-D114D3FBC4E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31365" yWindow="2355" windowWidth="21585" windowHeight="12645" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="9" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="69">
   <si>
     <t>ships</t>
   </si>
@@ -89,9 +89,6 @@
     <t>https://jgcri.github.io/gcam-doc/choice.html</t>
   </si>
   <si>
-    <t>Calibration</t>
-  </si>
-  <si>
     <t># File: A54.tranSubsector_logit_revised.csv</t>
   </si>
   <si>
@@ -230,13 +227,19 @@
     <t>2W</t>
   </si>
   <si>
-    <t>For non-road we use -0.1 because of costs preventing the model from solving.</t>
-  </si>
-  <si>
-    <t>We use calibrated values in onroad sectors.</t>
-  </si>
-  <si>
     <t>For more on this, see the "Unmodified Logit" equation description at:</t>
+  </si>
+  <si>
+    <t>PNNL</t>
+  </si>
+  <si>
+    <t>Global Change Analysis Model</t>
+  </si>
+  <si>
+    <t>https://github.com/JGCRI/gcam-core/tree/master/input/gcamdata/inst/extdata/energy</t>
+  </si>
+  <si>
+    <t>input &gt; gcamdata &gt; inst &gt; extdata &gt; energy &gt; A54.tranSubsector_logit_revised.csv</t>
   </si>
 </sst>
 </file>
@@ -247,7 +250,7 @@
     <numFmt numFmtId="164" formatCode="###0.00_)"/>
     <numFmt numFmtId="165" formatCode="#,##0_)"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1315,75 +1318,83 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B54"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="45.42578125" customWidth="1"/>
+    <col min="2" max="2" width="45.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="1"/>
+      <c r="B4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1"/>
+      <c r="B5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="1"/>
+      <c r="B6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
-      <c r="A10" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="54" spans="1:1">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" s="1"/>
     </row>
   </sheetData>
@@ -1395,415 +1406,415 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D97FB3F6-A063-4685-A6D1-3D6F2007ED8F}">
   <dimension ref="A1:E31"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="2" width="34.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.453125" customWidth="1"/>
+    <col min="2" max="2" width="34.1796875" customWidth="1"/>
+    <col min="3" max="3" width="14.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
         <v>25</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>27</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>28</v>
       </c>
-      <c r="E7" t="s">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
         <v>30</v>
-      </c>
-      <c r="B8" t="s">
-        <v>31</v>
       </c>
       <c r="C8">
         <v>-6</v>
       </c>
       <c r="E8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>33</v>
-      </c>
-      <c r="B9" t="s">
-        <v>34</v>
       </c>
       <c r="C9">
         <v>-6</v>
       </c>
       <c r="E9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" t="s">
-        <v>33</v>
-      </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C10">
         <v>-1</v>
       </c>
       <c r="D10" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>36</v>
       </c>
-      <c r="E10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
         <v>37</v>
-      </c>
-      <c r="B11" t="s">
-        <v>38</v>
       </c>
       <c r="C11">
         <v>-8</v>
       </c>
       <c r="D11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" t="s">
         <v>39</v>
-      </c>
-      <c r="E11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
-        <v>37</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
       </c>
       <c r="C12">
         <v>-8</v>
       </c>
       <c r="D12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E12" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C13">
         <v>-8</v>
       </c>
       <c r="D13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" t="s">
         <v>42</v>
-      </c>
-      <c r="B14" t="s">
-        <v>43</v>
       </c>
       <c r="C14">
         <v>-6</v>
       </c>
       <c r="E14" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15">
         <v>-6</v>
       </c>
       <c r="E15" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C16">
         <v>-6</v>
       </c>
       <c r="E16" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C17">
         <v>-1</v>
       </c>
       <c r="D17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E17" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C18">
         <v>-6</v>
       </c>
       <c r="E18" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" t="s">
         <v>48</v>
-      </c>
-      <c r="B19" t="s">
-        <v>49</v>
       </c>
       <c r="C19">
         <v>-3</v>
       </c>
       <c r="D19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E19" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" t="s">
         <v>50</v>
-      </c>
-      <c r="B20" t="s">
-        <v>51</v>
       </c>
       <c r="C20">
         <v>-8</v>
       </c>
       <c r="D20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E20" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
+        <v>51</v>
+      </c>
+      <c r="B21" t="s">
         <v>52</v>
-      </c>
-      <c r="B21" t="s">
-        <v>53</v>
       </c>
       <c r="C21">
         <v>-8</v>
       </c>
       <c r="D21" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" t="s">
         <v>54</v>
-      </c>
-      <c r="E21" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" t="s">
-        <v>52</v>
-      </c>
-      <c r="B22" t="s">
-        <v>55</v>
       </c>
       <c r="C22">
         <v>-8</v>
       </c>
       <c r="D22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E22" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
         <v>-8</v>
       </c>
       <c r="D23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E23" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" t="s">
         <v>57</v>
-      </c>
-      <c r="B24" t="s">
-        <v>58</v>
       </c>
       <c r="C24">
         <v>-6</v>
       </c>
       <c r="E24" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" t="s">
-        <v>42</v>
-      </c>
-      <c r="B26" t="s">
-        <v>60</v>
       </c>
       <c r="C26">
         <v>-6</v>
       </c>
       <c r="E26" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B27" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C27">
         <v>-6</v>
       </c>
       <c r="E27" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C28">
         <v>-6</v>
       </c>
       <c r="E28" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C29">
         <v>-6</v>
       </c>
       <c r="E29" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C30">
         <v>-6</v>
       </c>
       <c r="E30" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" t="s">
-        <v>33</v>
-      </c>
       <c r="B31" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C31">
         <v>-6</v>
       </c>
       <c r="E31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1817,14 +1828,14 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+    <col min="1" max="1" width="14.54296875" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -1835,70 +1846,82 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2">
-        <v>-80</v>
+        <f>'A54.tranSubsector_logit_revised'!C21</f>
+        <v>-8</v>
       </c>
       <c r="C2">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <f>'A54.tranSubsector_logit_revised'!C12</f>
+        <v>-8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3">
-        <v>-30</v>
+        <f>'A54.tranSubsector_logit_revised'!C19</f>
+        <v>-3</v>
       </c>
       <c r="C3">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+        <f>'A54.tranSubsector_logit_revised'!C13</f>
+        <v>-8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="B4">
-        <v>-0.1</v>
+        <f>'A54.tranSubsector_logit_revised'!C15</f>
+        <v>-6</v>
       </c>
       <c r="C4">
-        <v>-0.1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+        <f>B4</f>
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>1</v>
       </c>
       <c r="B5">
-        <v>-0.15</v>
+        <f>'A54.tranSubsector_logit_revised'!C17</f>
+        <v>-1</v>
       </c>
       <c r="C5">
-        <v>-0.1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <f>'A54.tranSubsector_logit_revised'!C10</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>0</v>
       </c>
       <c r="B6">
-        <v>-0.1</v>
+        <f>'A54.tranSubsector_logit_revised'!C9</f>
+        <v>-6</v>
       </c>
       <c r="C6">
-        <v>-0.1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+        <f>'A54.tranSubsector_logit_revised'!C24</f>
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>-40</v>
+        <f>'A54.tranSubsector_logit_revised'!C20</f>
+        <v>-8</v>
       </c>
       <c r="C7">
-        <v>-40</v>
+        <f>'A54.tranSubsector_logit_revised'!C20</f>
+        <v>-8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>